<commit_message>
Copied over Lab 5 code into Lab7 src directory and build locally successfully
</commit_message>
<xml_diff>
--- a/Lab7BOM.xlsx
+++ b/Lab7BOM.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="11004"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30527"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/harishthehershey/Desktop/HW/ECE 445L - TA/Golden/ECE445L-Lab7-10-Project/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/7d0bb276250f97ce/Documents/UT 2026-2027/ECE 445L/ece445l_lab7-10_fall26-4-ew-js-tp-ak/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8009E6A1-81EC-F24D-A862-C945870CFCFC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="3" documentId="13_ncr:1_{8009E6A1-81EC-F24D-A862-C945870CFCFC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{9F8947BF-4141-4772-9B42-C2F7AE20258B}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="660" windowWidth="30240" windowHeight="18980" xr2:uid="{2A746B91-5B93-4559-A98B-A0C4C3CDA5C8}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" xr2:uid="{2A746B91-5B93-4559-A98B-A0C4C3CDA5C8}"/>
   </bookViews>
   <sheets>
     <sheet name="Parts" sheetId="1" r:id="rId1"/>
@@ -2097,9 +2097,9 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4BB64E12-2F57-4D15-BA8D-127B966BFCD4}">
   <dimension ref="A1:R157"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="11.5" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr defaultColWidth="11.44140625" defaultRowHeight="15.6" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="9.1640625" style="3" customWidth="1"/>
+    <col min="1" max="1" width="9.109375" style="3" customWidth="1"/>
     <col min="2" max="3" width="11.33203125" style="3" customWidth="1"/>
     <col min="4" max="4" width="46.6640625" style="3" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="25" style="3" customWidth="1"/>
@@ -2107,11 +2107,11 @@
     <col min="7" max="7" width="18" style="3" bestFit="1" customWidth="1"/>
     <col min="8" max="8" width="24.6640625" style="3" customWidth="1"/>
     <col min="9" max="9" width="9.33203125" style="2" customWidth="1"/>
-    <col min="10" max="10" width="9.1640625" style="2" customWidth="1"/>
-    <col min="11" max="16384" width="11.5" style="1"/>
+    <col min="10" max="10" width="12.44140625" style="2" customWidth="1"/>
+    <col min="11" max="16384" width="11.44140625" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A1" s="6" t="s">
         <v>5</v>
       </c>
@@ -2129,7 +2129,7 @@
       </c>
       <c r="H1" s="6"/>
     </row>
-    <row r="2" spans="1:12" ht="19" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:12" ht="18" x14ac:dyDescent="0.35">
       <c r="A2" s="6" t="s">
         <v>463</v>
       </c>
@@ -2145,7 +2145,7 @@
       <c r="G2" s="6"/>
       <c r="H2" s="6"/>
     </row>
-    <row r="3" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A3" s="6"/>
       <c r="B3" s="6"/>
       <c r="C3" s="6"/>
@@ -2157,7 +2157,7 @@
       <c r="G3" s="6"/>
       <c r="H3" s="6"/>
     </row>
-    <row r="4" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A4" s="3" t="s">
         <v>236</v>
       </c>
@@ -2168,7 +2168,7 @@
         <v>452</v>
       </c>
     </row>
-    <row r="5" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A5" s="3" t="s">
         <v>0</v>
       </c>
@@ -2206,9 +2206,9 @@
         <v>238</v>
       </c>
     </row>
-    <row r="6" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A6" s="3">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="C6" s="3" t="s">
         <v>28</v>
@@ -2221,14 +2221,14 @@
       </c>
       <c r="J6" s="2">
         <f t="shared" ref="J6:J35" si="0">A6*I6</f>
-        <v>0</v>
+        <v>0.6</v>
       </c>
       <c r="K6" s="1" t="s">
         <v>447</v>
       </c>
       <c r="L6" s="5"/>
     </row>
-    <row r="7" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A7" s="3">
         <v>0</v>
       </c>
@@ -2249,7 +2249,7 @@
         <v>241</v>
       </c>
     </row>
-    <row r="8" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A8" s="3">
         <v>0</v>
       </c>
@@ -2285,7 +2285,7 @@
         <v>306</v>
       </c>
     </row>
-    <row r="9" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="9" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A9" s="3">
         <v>0</v>
       </c>
@@ -2309,7 +2309,7 @@
         <v>242</v>
       </c>
     </row>
-    <row r="10" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="10" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A10" s="3">
         <v>0</v>
       </c>
@@ -2336,7 +2336,7 @@
         <v>242</v>
       </c>
     </row>
-    <row r="11" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="11" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A11" s="3">
         <v>0</v>
       </c>
@@ -2369,7 +2369,7 @@
         <v>242</v>
       </c>
     </row>
-    <row r="12" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="12" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A12" s="3">
         <v>0</v>
       </c>
@@ -2396,7 +2396,7 @@
         <v>242</v>
       </c>
     </row>
-    <row r="13" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="13" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A13" s="3">
         <v>0</v>
       </c>
@@ -2423,7 +2423,7 @@
         <v>242</v>
       </c>
     </row>
-    <row r="14" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="14" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A14" s="3">
         <v>0</v>
       </c>
@@ -2444,7 +2444,7 @@
         <v>242</v>
       </c>
     </row>
-    <row r="15" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="15" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A15" s="3">
         <v>0</v>
       </c>
@@ -2471,7 +2471,7 @@
         <v>242</v>
       </c>
     </row>
-    <row r="16" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="16" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A16" s="3">
         <v>0</v>
       </c>
@@ -2498,7 +2498,7 @@
         <v>242</v>
       </c>
     </row>
-    <row r="17" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="17" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A17" s="3">
         <v>0</v>
       </c>
@@ -2519,7 +2519,7 @@
         <v>242</v>
       </c>
     </row>
-    <row r="18" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="18" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A18" s="3">
         <v>0</v>
       </c>
@@ -2540,7 +2540,7 @@
         <v>242</v>
       </c>
     </row>
-    <row r="19" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="19" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A19" s="3">
         <v>0</v>
       </c>
@@ -2561,7 +2561,7 @@
         <v>242</v>
       </c>
     </row>
-    <row r="20" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="20" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A20" s="3">
         <v>0</v>
       </c>
@@ -2582,7 +2582,7 @@
         <v>242</v>
       </c>
     </row>
-    <row r="21" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="21" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A21" s="3">
         <v>0</v>
       </c>
@@ -2603,7 +2603,7 @@
         <v>242</v>
       </c>
     </row>
-    <row r="22" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="22" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A22" s="3">
         <v>0</v>
       </c>
@@ -2624,7 +2624,7 @@
         <v>242</v>
       </c>
     </row>
-    <row r="23" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="23" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A23" s="3">
         <v>0</v>
       </c>
@@ -2651,7 +2651,7 @@
         <v>242</v>
       </c>
     </row>
-    <row r="24" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="24" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A24" s="3">
         <v>0</v>
       </c>
@@ -2684,7 +2684,7 @@
         <v>242</v>
       </c>
     </row>
-    <row r="25" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="25" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A25" s="3">
         <v>0</v>
       </c>
@@ -2717,7 +2717,7 @@
         <v>242</v>
       </c>
     </row>
-    <row r="26" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="26" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A26" s="3">
         <v>0</v>
       </c>
@@ -2744,7 +2744,7 @@
         <v>242</v>
       </c>
     </row>
-    <row r="27" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="27" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A27" s="3">
         <v>0</v>
       </c>
@@ -2771,7 +2771,7 @@
         <v>242</v>
       </c>
     </row>
-    <row r="28" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="28" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A28" s="3">
         <v>0</v>
       </c>
@@ -2798,7 +2798,7 @@
         <v>242</v>
       </c>
     </row>
-    <row r="29" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="29" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A29" s="3">
         <v>0</v>
       </c>
@@ -2825,7 +2825,7 @@
         <v>242</v>
       </c>
     </row>
-    <row r="30" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="30" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A30" s="3">
         <v>0</v>
       </c>
@@ -2852,7 +2852,7 @@
         <v>242</v>
       </c>
     </row>
-    <row r="31" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="31" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A31" s="3">
         <v>0</v>
       </c>
@@ -2879,7 +2879,7 @@
         <v>242</v>
       </c>
     </row>
-    <row r="32" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="32" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A32" s="3">
         <v>0</v>
       </c>
@@ -2906,7 +2906,7 @@
         <v>242</v>
       </c>
     </row>
-    <row r="33" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="33" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A33" s="3">
         <v>0</v>
       </c>
@@ -2933,7 +2933,7 @@
         <v>242</v>
       </c>
     </row>
-    <row r="34" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="34" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A34" s="3">
         <v>0</v>
       </c>
@@ -2960,7 +2960,7 @@
         <v>242</v>
       </c>
     </row>
-    <row r="35" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="35" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A35" s="3">
         <v>0</v>
       </c>
@@ -2993,7 +2993,7 @@
         <v>242</v>
       </c>
     </row>
-    <row r="36" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="36" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A36" s="3">
         <v>0</v>
       </c>
@@ -3026,7 +3026,7 @@
         <v>242</v>
       </c>
     </row>
-    <row r="37" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="37" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A37" s="3">
         <v>0</v>
       </c>
@@ -3059,7 +3059,7 @@
         <v>242</v>
       </c>
     </row>
-    <row r="38" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="38" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A38" s="3">
         <v>0</v>
       </c>
@@ -3092,7 +3092,7 @@
         <v>242</v>
       </c>
     </row>
-    <row r="39" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="39" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A39" s="3">
         <v>0</v>
       </c>
@@ -3125,7 +3125,7 @@
         <v>242</v>
       </c>
     </row>
-    <row r="40" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="40" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A40" s="3">
         <v>0</v>
       </c>
@@ -3158,7 +3158,7 @@
         <v>242</v>
       </c>
     </row>
-    <row r="41" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="41" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A41" s="3">
         <v>0</v>
       </c>
@@ -3191,7 +3191,7 @@
         <v>242</v>
       </c>
     </row>
-    <row r="42" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="42" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A42" s="3">
         <v>0</v>
       </c>
@@ -3218,7 +3218,7 @@
         <v>242</v>
       </c>
     </row>
-    <row r="43" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="43" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A43" s="3">
         <v>0</v>
       </c>
@@ -3245,7 +3245,7 @@
         <v>242</v>
       </c>
     </row>
-    <row r="44" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="44" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A44" s="3">
         <v>0</v>
       </c>
@@ -3272,7 +3272,7 @@
         <v>242</v>
       </c>
     </row>
-    <row r="45" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="45" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A45" s="3">
         <v>0</v>
       </c>
@@ -3299,7 +3299,7 @@
         <v>242</v>
       </c>
     </row>
-    <row r="46" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="46" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A46" s="3">
         <v>0</v>
       </c>
@@ -3335,7 +3335,7 @@
         <v>352</v>
       </c>
     </row>
-    <row r="47" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="47" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A47" s="3">
         <v>0</v>
       </c>
@@ -3368,7 +3368,7 @@
         <v>242</v>
       </c>
     </row>
-    <row r="48" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="48" spans="1:12" x14ac:dyDescent="0.3">
       <c r="C48" s="3" t="s">
         <v>30</v>
       </c>
@@ -3398,7 +3398,7 @@
         <v>242</v>
       </c>
     </row>
-    <row r="49" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="49" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A49" s="3">
         <v>0</v>
       </c>
@@ -3431,7 +3431,7 @@
         <v>242</v>
       </c>
     </row>
-    <row r="50" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="50" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A50" s="3">
         <v>0</v>
       </c>
@@ -3464,7 +3464,7 @@
         <v>242</v>
       </c>
     </row>
-    <row r="51" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="51" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A51" s="3">
         <v>0</v>
       </c>
@@ -3497,7 +3497,7 @@
         <v>242</v>
       </c>
     </row>
-    <row r="52" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="52" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A52" s="3">
         <v>0</v>
       </c>
@@ -3518,7 +3518,7 @@
         <v>242</v>
       </c>
     </row>
-    <row r="53" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="53" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A53" s="3">
         <v>0</v>
       </c>
@@ -3548,7 +3548,7 @@
         <v>242</v>
       </c>
     </row>
-    <row r="54" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="54" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A54" s="3">
         <v>0</v>
       </c>
@@ -3575,7 +3575,7 @@
         <v>242</v>
       </c>
     </row>
-    <row r="55" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="55" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A55" s="3">
         <v>0</v>
       </c>
@@ -3608,7 +3608,7 @@
         <v>448</v>
       </c>
     </row>
-    <row r="56" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="56" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A56" s="3">
         <v>0</v>
       </c>
@@ -3644,7 +3644,7 @@
         <v>448</v>
       </c>
     </row>
-    <row r="57" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="57" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A57" s="3">
         <v>0</v>
       </c>
@@ -3677,7 +3677,7 @@
         <v>242</v>
       </c>
     </row>
-    <row r="58" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="58" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A58" s="3">
         <v>0</v>
       </c>
@@ -3710,7 +3710,7 @@
         <v>447</v>
       </c>
     </row>
-    <row r="59" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="59" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A59" s="3">
         <v>0</v>
       </c>
@@ -3743,7 +3743,7 @@
         <v>242</v>
       </c>
     </row>
-    <row r="60" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="60" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A60" s="3">
         <v>0</v>
       </c>
@@ -3776,7 +3776,7 @@
         <v>242</v>
       </c>
     </row>
-    <row r="61" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="61" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A61" s="3">
         <v>0</v>
       </c>
@@ -3809,7 +3809,7 @@
         <v>242</v>
       </c>
     </row>
-    <row r="62" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="62" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A62" s="3">
         <v>0</v>
       </c>
@@ -3836,7 +3836,7 @@
         <v>224</v>
       </c>
     </row>
-    <row r="63" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="63" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A63" s="3">
         <v>0</v>
       </c>
@@ -3866,7 +3866,7 @@
         <v>440</v>
       </c>
     </row>
-    <row r="64" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="64" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A64" s="3">
         <v>0</v>
       </c>
@@ -3896,7 +3896,7 @@
         <v>224</v>
       </c>
     </row>
-    <row r="65" spans="1:18" x14ac:dyDescent="0.2">
+    <row r="65" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A65" s="3">
         <v>0</v>
       </c>
@@ -3926,7 +3926,7 @@
         <v>224</v>
       </c>
     </row>
-    <row r="66" spans="1:18" x14ac:dyDescent="0.2">
+    <row r="66" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A66" s="3">
         <v>0</v>
       </c>
@@ -3956,7 +3956,7 @@
         <v>224</v>
       </c>
     </row>
-    <row r="67" spans="1:18" x14ac:dyDescent="0.2">
+    <row r="67" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A67" s="3">
         <v>0</v>
       </c>
@@ -3986,7 +3986,7 @@
         <v>440</v>
       </c>
     </row>
-    <row r="68" spans="1:18" x14ac:dyDescent="0.2">
+    <row r="68" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A68" s="3">
         <v>0</v>
       </c>
@@ -4019,7 +4019,7 @@
         <v>250</v>
       </c>
     </row>
-    <row r="69" spans="1:18" x14ac:dyDescent="0.2">
+    <row r="69" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A69" s="3">
         <v>0</v>
       </c>
@@ -4055,7 +4055,7 @@
         <v>251</v>
       </c>
     </row>
-    <row r="70" spans="1:18" x14ac:dyDescent="0.2">
+    <row r="70" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A70" s="3">
         <v>0</v>
       </c>
@@ -4091,7 +4091,7 @@
         <v>252</v>
       </c>
     </row>
-    <row r="71" spans="1:18" x14ac:dyDescent="0.2">
+    <row r="71" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A71" s="3">
         <v>0</v>
       </c>
@@ -4127,7 +4127,7 @@
         <v>253</v>
       </c>
     </row>
-    <row r="72" spans="1:18" x14ac:dyDescent="0.2">
+    <row r="72" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A72" s="3">
         <v>0</v>
       </c>
@@ -4163,7 +4163,7 @@
         <v>254</v>
       </c>
     </row>
-    <row r="73" spans="1:18" x14ac:dyDescent="0.2">
+    <row r="73" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A73" s="3">
         <v>0</v>
       </c>
@@ -4199,7 +4199,7 @@
         <v>255</v>
       </c>
     </row>
-    <row r="74" spans="1:18" x14ac:dyDescent="0.2">
+    <row r="74" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A74" s="3">
         <v>0</v>
       </c>
@@ -4235,7 +4235,7 @@
         <v>256</v>
       </c>
     </row>
-    <row r="75" spans="1:18" x14ac:dyDescent="0.2">
+    <row r="75" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A75" s="3">
         <v>0</v>
       </c>
@@ -4255,7 +4255,7 @@
         <v>184</v>
       </c>
     </row>
-    <row r="76" spans="1:18" x14ac:dyDescent="0.2">
+    <row r="76" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A76" s="3">
         <v>0</v>
       </c>
@@ -4285,7 +4285,7 @@
         <v>257</v>
       </c>
     </row>
-    <row r="77" spans="1:18" x14ac:dyDescent="0.2">
+    <row r="77" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A77" s="3">
         <v>0</v>
       </c>
@@ -4315,7 +4315,7 @@
         <v>258</v>
       </c>
     </row>
-    <row r="78" spans="1:18" x14ac:dyDescent="0.2">
+    <row r="78" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A78" s="3">
         <v>0</v>
       </c>
@@ -4351,7 +4351,7 @@
         <v>258</v>
       </c>
     </row>
-    <row r="79" spans="1:18" x14ac:dyDescent="0.2">
+    <row r="79" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A79" s="3">
         <v>0</v>
       </c>
@@ -4387,7 +4387,7 @@
         <v>259</v>
       </c>
     </row>
-    <row r="80" spans="1:18" x14ac:dyDescent="0.2">
+    <row r="80" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A80" s="3">
         <v>0</v>
       </c>
@@ -4417,7 +4417,7 @@
         <v>260</v>
       </c>
     </row>
-    <row r="81" spans="1:17" x14ac:dyDescent="0.2">
+    <row r="81" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A81" s="3">
         <v>0</v>
       </c>
@@ -4447,7 +4447,7 @@
         <v>249</v>
       </c>
     </row>
-    <row r="82" spans="1:17" x14ac:dyDescent="0.2">
+    <row r="82" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A82" s="3">
         <v>0</v>
       </c>
@@ -4483,7 +4483,7 @@
         <v>196</v>
       </c>
     </row>
-    <row r="83" spans="1:17" x14ac:dyDescent="0.2">
+    <row r="83" spans="1:17" x14ac:dyDescent="0.3">
       <c r="C83" s="3" t="s">
         <v>33</v>
       </c>
@@ -4513,7 +4513,7 @@
         <v>195</v>
       </c>
     </row>
-    <row r="84" spans="1:17" x14ac:dyDescent="0.2">
+    <row r="84" spans="1:17" x14ac:dyDescent="0.3">
       <c r="C84" s="3" t="s">
         <v>33</v>
       </c>
@@ -4543,7 +4543,7 @@
         <v>195</v>
       </c>
     </row>
-    <row r="85" spans="1:17" x14ac:dyDescent="0.2">
+    <row r="85" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A85" s="3">
         <v>0</v>
       </c>
@@ -4576,7 +4576,7 @@
         <v>242</v>
       </c>
     </row>
-    <row r="86" spans="1:17" x14ac:dyDescent="0.2">
+    <row r="86" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A86" s="3">
         <v>0</v>
       </c>
@@ -4609,7 +4609,7 @@
         <v>242</v>
       </c>
     </row>
-    <row r="87" spans="1:17" x14ac:dyDescent="0.2">
+    <row r="87" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A87" s="3">
         <v>0</v>
       </c>
@@ -4642,7 +4642,7 @@
         <v>242</v>
       </c>
     </row>
-    <row r="88" spans="1:17" x14ac:dyDescent="0.2">
+    <row r="88" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A88" s="3">
         <v>0</v>
       </c>
@@ -4675,7 +4675,7 @@
         <v>242</v>
       </c>
     </row>
-    <row r="89" spans="1:17" x14ac:dyDescent="0.2">
+    <row r="89" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A89" s="3">
         <v>0</v>
       </c>
@@ -4699,7 +4699,7 @@
         <v>312</v>
       </c>
     </row>
-    <row r="90" spans="1:17" x14ac:dyDescent="0.2">
+    <row r="90" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A90" s="3">
         <v>0</v>
       </c>
@@ -4726,7 +4726,7 @@
         <v>231</v>
       </c>
     </row>
-    <row r="91" spans="1:17" x14ac:dyDescent="0.2">
+    <row r="91" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A91" s="3">
         <v>0</v>
       </c>
@@ -4747,7 +4747,7 @@
         <v>447</v>
       </c>
     </row>
-    <row r="92" spans="1:17" x14ac:dyDescent="0.2">
+    <row r="92" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A92" s="3">
         <v>0</v>
       </c>
@@ -4768,7 +4768,7 @@
         <v>242</v>
       </c>
     </row>
-    <row r="93" spans="1:17" x14ac:dyDescent="0.2">
+    <row r="93" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A93" s="3">
         <v>0</v>
       </c>
@@ -4789,7 +4789,7 @@
         <v>242</v>
       </c>
     </row>
-    <row r="94" spans="1:17" x14ac:dyDescent="0.2">
+    <row r="94" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A94" s="3">
         <v>0</v>
       </c>
@@ -4822,7 +4822,7 @@
         <v>242</v>
       </c>
     </row>
-    <row r="95" spans="1:17" x14ac:dyDescent="0.2">
+    <row r="95" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A95" s="3">
         <v>0</v>
       </c>
@@ -4855,7 +4855,7 @@
         <v>242</v>
       </c>
     </row>
-    <row r="96" spans="1:17" x14ac:dyDescent="0.2">
+    <row r="96" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A96" s="3">
         <v>0</v>
       </c>
@@ -4888,7 +4888,7 @@
         <v>242</v>
       </c>
     </row>
-    <row r="97" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="97" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A97" s="3">
         <v>0</v>
       </c>
@@ -4921,7 +4921,7 @@
         <v>242</v>
       </c>
     </row>
-    <row r="98" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="98" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A98" s="3">
         <v>0</v>
       </c>
@@ -4954,7 +4954,7 @@
         <v>242</v>
       </c>
     </row>
-    <row r="99" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="99" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A99" s="3">
         <v>0</v>
       </c>
@@ -4987,7 +4987,7 @@
         <v>242</v>
       </c>
     </row>
-    <row r="100" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="100" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A100" s="3">
         <v>0</v>
       </c>
@@ -5020,7 +5020,7 @@
         <v>242</v>
       </c>
     </row>
-    <row r="101" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="101" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A101" s="3">
         <v>0</v>
       </c>
@@ -5053,7 +5053,7 @@
         <v>242</v>
       </c>
     </row>
-    <row r="102" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="102" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A102" s="3">
         <v>0</v>
       </c>
@@ -5086,7 +5086,7 @@
         <v>242</v>
       </c>
     </row>
-    <row r="103" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="103" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A103" s="3">
         <v>0</v>
       </c>
@@ -5119,7 +5119,7 @@
         <v>242</v>
       </c>
     </row>
-    <row r="104" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="104" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A104" s="3">
         <v>0</v>
       </c>
@@ -5152,7 +5152,7 @@
         <v>242</v>
       </c>
     </row>
-    <row r="105" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="105" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A105" s="3">
         <v>0</v>
       </c>
@@ -5185,7 +5185,7 @@
         <v>242</v>
       </c>
     </row>
-    <row r="106" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="106" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A106" s="3">
         <v>0</v>
       </c>
@@ -5218,7 +5218,7 @@
         <v>242</v>
       </c>
     </row>
-    <row r="107" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="107" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A107" s="3">
         <v>0</v>
       </c>
@@ -5251,7 +5251,7 @@
         <v>242</v>
       </c>
     </row>
-    <row r="108" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="108" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A108" s="3">
         <v>0</v>
       </c>
@@ -5284,7 +5284,7 @@
         <v>242</v>
       </c>
     </row>
-    <row r="109" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="109" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A109" s="3">
         <v>0</v>
       </c>
@@ -5317,7 +5317,7 @@
         <v>242</v>
       </c>
     </row>
-    <row r="110" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="110" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A110" s="3">
         <v>0</v>
       </c>
@@ -5350,7 +5350,7 @@
         <v>242</v>
       </c>
     </row>
-    <row r="111" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="111" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A111" s="3">
         <v>0</v>
       </c>
@@ -5383,7 +5383,7 @@
         <v>242</v>
       </c>
     </row>
-    <row r="112" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="112" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A112" s="3">
         <v>0</v>
       </c>
@@ -5416,7 +5416,7 @@
         <v>242</v>
       </c>
     </row>
-    <row r="113" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="113" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A113" s="3">
         <v>0</v>
       </c>
@@ -5449,7 +5449,7 @@
         <v>242</v>
       </c>
     </row>
-    <row r="114" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="114" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A114" s="3">
         <v>0</v>
       </c>
@@ -5482,7 +5482,7 @@
         <v>242</v>
       </c>
     </row>
-    <row r="115" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="115" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A115" s="3">
         <v>0</v>
       </c>
@@ -5515,7 +5515,7 @@
         <v>242</v>
       </c>
     </row>
-    <row r="116" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="116" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A116" s="3">
         <v>0</v>
       </c>
@@ -5548,7 +5548,7 @@
         <v>242</v>
       </c>
     </row>
-    <row r="117" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="117" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A117" s="3">
         <v>0</v>
       </c>
@@ -5581,7 +5581,7 @@
         <v>242</v>
       </c>
     </row>
-    <row r="118" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="118" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A118" s="3">
         <v>0</v>
       </c>
@@ -5617,7 +5617,7 @@
         <v>164</v>
       </c>
     </row>
-    <row r="119" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="119" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A119" s="3">
         <v>0</v>
       </c>
@@ -5650,7 +5650,7 @@
         <v>242</v>
       </c>
     </row>
-    <row r="120" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="120" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A120" s="3">
         <v>0</v>
       </c>
@@ -5683,7 +5683,7 @@
         <v>242</v>
       </c>
     </row>
-    <row r="121" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="121" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A121" s="3">
         <v>0</v>
       </c>
@@ -5716,7 +5716,7 @@
         <v>242</v>
       </c>
     </row>
-    <row r="122" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="122" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A122" s="3">
         <v>0</v>
       </c>
@@ -5749,7 +5749,7 @@
         <v>242</v>
       </c>
     </row>
-    <row r="123" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="123" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A123" s="3">
         <v>0</v>
       </c>
@@ -5782,7 +5782,7 @@
         <v>242</v>
       </c>
     </row>
-    <row r="124" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="124" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A124" s="3">
         <v>0</v>
       </c>
@@ -5815,7 +5815,7 @@
         <v>242</v>
       </c>
     </row>
-    <row r="125" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="125" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A125" s="3">
         <v>0</v>
       </c>
@@ -5848,7 +5848,7 @@
         <v>242</v>
       </c>
     </row>
-    <row r="126" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="126" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A126" s="3">
         <v>0</v>
       </c>
@@ -5881,7 +5881,7 @@
         <v>242</v>
       </c>
     </row>
-    <row r="127" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="127" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A127" s="3">
         <v>0</v>
       </c>
@@ -5914,7 +5914,7 @@
         <v>242</v>
       </c>
     </row>
-    <row r="128" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="128" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A128" s="3">
         <v>0</v>
       </c>
@@ -5947,7 +5947,7 @@
         <v>242</v>
       </c>
     </row>
-    <row r="129" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="129" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A129" s="3">
         <v>0</v>
       </c>
@@ -5980,7 +5980,7 @@
         <v>242</v>
       </c>
     </row>
-    <row r="130" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="130" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A130" s="3">
         <v>0</v>
       </c>
@@ -6013,7 +6013,7 @@
         <v>242</v>
       </c>
     </row>
-    <row r="131" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="131" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A131" s="3">
         <v>0</v>
       </c>
@@ -6046,7 +6046,7 @@
         <v>242</v>
       </c>
     </row>
-    <row r="132" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="132" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A132" s="3">
         <v>0</v>
       </c>
@@ -6079,7 +6079,7 @@
         <v>242</v>
       </c>
     </row>
-    <row r="133" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="133" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A133" s="3">
         <v>0</v>
       </c>
@@ -6112,7 +6112,7 @@
         <v>242</v>
       </c>
     </row>
-    <row r="134" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="134" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A134" s="3">
         <v>0</v>
       </c>
@@ -6145,7 +6145,7 @@
         <v>242</v>
       </c>
     </row>
-    <row r="135" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="135" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A135" s="3">
         <v>0</v>
       </c>
@@ -6178,7 +6178,7 @@
         <v>242</v>
       </c>
     </row>
-    <row r="136" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="136" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A136" s="3">
         <v>0</v>
       </c>
@@ -6211,7 +6211,7 @@
         <v>242</v>
       </c>
     </row>
-    <row r="137" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="137" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A137" s="3">
         <v>0</v>
       </c>
@@ -6244,7 +6244,7 @@
         <v>242</v>
       </c>
     </row>
-    <row r="138" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="138" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A138" s="3">
         <v>0</v>
       </c>
@@ -6277,7 +6277,7 @@
         <v>242</v>
       </c>
     </row>
-    <row r="139" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="139" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A139" s="3">
         <v>0</v>
       </c>
@@ -6310,7 +6310,7 @@
         <v>242</v>
       </c>
     </row>
-    <row r="140" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="140" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A140" s="3">
         <v>0</v>
       </c>
@@ -6343,7 +6343,7 @@
         <v>242</v>
       </c>
     </row>
-    <row r="141" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="141" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A141" s="3">
         <v>0</v>
       </c>
@@ -6376,7 +6376,7 @@
         <v>242</v>
       </c>
     </row>
-    <row r="142" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="142" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A142" s="3">
         <v>0</v>
       </c>
@@ -6409,7 +6409,7 @@
         <v>242</v>
       </c>
     </row>
-    <row r="143" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="143" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A143" s="3">
         <v>0</v>
       </c>
@@ -6442,7 +6442,7 @@
         <v>242</v>
       </c>
     </row>
-    <row r="144" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="144" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A144" s="3">
         <v>0</v>
       </c>
@@ -6475,7 +6475,7 @@
         <v>242</v>
       </c>
     </row>
-    <row r="145" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="145" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A145" s="3">
         <v>0</v>
       </c>
@@ -6508,7 +6508,7 @@
         <v>242</v>
       </c>
     </row>
-    <row r="146" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="146" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A146" s="3">
         <v>0</v>
       </c>
@@ -6541,7 +6541,7 @@
         <v>242</v>
       </c>
     </row>
-    <row r="147" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="147" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A147" s="3">
         <v>0</v>
       </c>
@@ -6574,7 +6574,7 @@
         <v>242</v>
       </c>
     </row>
-    <row r="148" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="148" spans="1:12" x14ac:dyDescent="0.3">
       <c r="C148" s="3" t="s">
         <v>38</v>
       </c>
@@ -6604,7 +6604,7 @@
         <v>242</v>
       </c>
     </row>
-    <row r="149" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="149" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A149" s="3">
         <v>0</v>
       </c>
@@ -6637,7 +6637,7 @@
         <v>242</v>
       </c>
     </row>
-    <row r="150" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="150" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A150" s="3">
         <v>0</v>
       </c>
@@ -6658,7 +6658,7 @@
         <v>242</v>
       </c>
     </row>
-    <row r="151" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="151" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A151" s="3">
         <v>0</v>
       </c>
@@ -6679,7 +6679,7 @@
         <v>242</v>
       </c>
     </row>
-    <row r="152" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="152" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A152" s="3">
         <v>0</v>
       </c>
@@ -6706,7 +6706,7 @@
         <v>242</v>
       </c>
     </row>
-    <row r="153" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="153" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A153" s="3">
         <v>0</v>
       </c>
@@ -6742,7 +6742,7 @@
         <v>358</v>
       </c>
     </row>
-    <row r="154" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="154" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A154" s="3">
         <v>0</v>
       </c>
@@ -6775,7 +6775,7 @@
         <v>242</v>
       </c>
     </row>
-    <row r="155" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="155" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A155" s="3">
         <v>0</v>
       </c>
@@ -6808,7 +6808,7 @@
         <v>242</v>
       </c>
     </row>
-    <row r="156" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="156" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A156" s="3">
         <v>0</v>
       </c>
@@ -6838,7 +6838,7 @@
         <v>447</v>
       </c>
     </row>
-    <row r="157" spans="1:12" ht="17" x14ac:dyDescent="0.2">
+    <row r="157" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A157" s="3">
         <v>0</v>
       </c>
@@ -6889,128 +6889,128 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0F259CE0-00F5-4859-8537-F4B5EB7CD0DC}">
   <dimension ref="A1:E18"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="13" x14ac:dyDescent="0.15"/>
+  <sheetFormatPr defaultColWidth="8.77734375" defaultRowHeight="13.2" x14ac:dyDescent="0.25"/>
   <sheetData>
-    <row r="1" spans="1:5" ht="16" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:5" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A1" s="3"/>
       <c r="B1" s="1"/>
       <c r="C1" s="1"/>
       <c r="D1" s="3"/>
       <c r="E1" s="1"/>
     </row>
-    <row r="2" spans="1:5" ht="16" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:5" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A2" s="3"/>
       <c r="B2" s="1"/>
       <c r="C2" s="1"/>
       <c r="D2" s="3"/>
       <c r="E2" s="1"/>
     </row>
-    <row r="3" spans="1:5" ht="16" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:5" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A3" s="3"/>
       <c r="B3" s="1"/>
       <c r="C3" s="1"/>
       <c r="D3" s="3"/>
       <c r="E3" s="1"/>
     </row>
-    <row r="4" spans="1:5" ht="16" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:5" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A4" s="3"/>
       <c r="B4" s="1"/>
       <c r="C4" s="1"/>
       <c r="D4" s="3"/>
       <c r="E4" s="1"/>
     </row>
-    <row r="5" spans="1:5" ht="16" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:5" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A5" s="3"/>
       <c r="B5" s="1"/>
       <c r="C5" s="1"/>
       <c r="D5" s="3"/>
       <c r="E5" s="1"/>
     </row>
-    <row r="6" spans="1:5" ht="16" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:5" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A6" s="3"/>
       <c r="B6" s="1"/>
       <c r="C6" s="1"/>
       <c r="D6" s="3"/>
       <c r="E6" s="1"/>
     </row>
-    <row r="7" spans="1:5" ht="16" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:5" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A7" s="3"/>
       <c r="B7" s="1"/>
       <c r="C7" s="1"/>
       <c r="D7" s="3"/>
       <c r="E7" s="1"/>
     </row>
-    <row r="8" spans="1:5" ht="16" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:5" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A8" s="3"/>
       <c r="B8" s="1"/>
       <c r="C8" s="1"/>
       <c r="D8" s="3"/>
       <c r="E8" s="1"/>
     </row>
-    <row r="9" spans="1:5" ht="16" x14ac:dyDescent="0.2">
+    <row r="9" spans="1:5" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A9" s="3"/>
       <c r="B9" s="1"/>
       <c r="C9" s="1"/>
       <c r="D9" s="3"/>
       <c r="E9" s="1"/>
     </row>
-    <row r="10" spans="1:5" ht="16" x14ac:dyDescent="0.2">
+    <row r="10" spans="1:5" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A10" s="3"/>
       <c r="B10" s="1"/>
       <c r="C10" s="1"/>
       <c r="D10" s="3"/>
       <c r="E10" s="1"/>
     </row>
-    <row r="11" spans="1:5" ht="16" x14ac:dyDescent="0.2">
+    <row r="11" spans="1:5" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A11" s="3"/>
       <c r="B11" s="1"/>
       <c r="C11" s="1"/>
       <c r="D11" s="3"/>
       <c r="E11" s="1"/>
     </row>
-    <row r="12" spans="1:5" ht="16" x14ac:dyDescent="0.2">
+    <row r="12" spans="1:5" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A12" s="3"/>
       <c r="B12" s="1"/>
       <c r="C12" s="1"/>
       <c r="D12" s="3"/>
       <c r="E12" s="1"/>
     </row>
-    <row r="13" spans="1:5" ht="16" x14ac:dyDescent="0.2">
+    <row r="13" spans="1:5" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A13" s="3"/>
       <c r="B13" s="1"/>
       <c r="C13" s="1"/>
       <c r="D13" s="3"/>
       <c r="E13" s="1"/>
     </row>
-    <row r="14" spans="1:5" ht="16" x14ac:dyDescent="0.2">
+    <row r="14" spans="1:5" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A14" s="3"/>
       <c r="B14" s="1"/>
       <c r="C14" s="1"/>
       <c r="D14" s="3"/>
       <c r="E14" s="1"/>
     </row>
-    <row r="15" spans="1:5" ht="16" x14ac:dyDescent="0.2">
+    <row r="15" spans="1:5" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A15" s="3"/>
       <c r="B15" s="1"/>
       <c r="C15" s="1"/>
       <c r="D15" s="3"/>
       <c r="E15" s="1"/>
     </row>
-    <row r="16" spans="1:5" ht="16" x14ac:dyDescent="0.2">
+    <row r="16" spans="1:5" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A16" s="3"/>
       <c r="B16" s="1"/>
       <c r="C16" s="1"/>
       <c r="D16" s="3"/>
       <c r="E16" s="1"/>
     </row>
-    <row r="17" spans="1:5" ht="16" x14ac:dyDescent="0.2">
+    <row r="17" spans="1:5" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A17" s="3"/>
       <c r="B17" s="1"/>
       <c r="C17" s="1"/>
       <c r="D17" s="3"/>
       <c r="E17" s="1"/>
     </row>
-    <row r="18" spans="1:5" ht="16" x14ac:dyDescent="0.2">
+    <row r="18" spans="1:5" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A18" s="3"/>
       <c r="B18" s="1"/>
       <c r="C18" s="1"/>

</xml_diff>

<commit_message>
Updated lab report and started the bom a little
</commit_message>
<xml_diff>
--- a/Lab7BOM.xlsx
+++ b/Lab7BOM.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/7d0bb276250f97ce/Documents/UT 2026-2027/ECE 445L/ece445l_lab7-10_fall26-4-ew-js-tp-ak/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="3" documentId="13_ncr:1_{8009E6A1-81EC-F24D-A862-C945870CFCFC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{9F8947BF-4141-4772-9B42-C2F7AE20258B}"/>
+  <xr:revisionPtr revIDLastSave="14" documentId="13_ncr:1_{8009E6A1-81EC-F24D-A862-C945870CFCFC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{6BA76F47-4657-418C-ABF7-4E570B270324}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" xr2:uid="{2A746B91-5B93-4559-A98B-A0C4C3CDA5C8}"/>
   </bookViews>
@@ -96,7 +96,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="965" uniqueCount="464">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="972" uniqueCount="467">
   <si>
     <t>Quantity</t>
   </si>
@@ -1530,6 +1530,15 @@
   </si>
   <si>
     <t>ECE445L Fall 2026</t>
+  </si>
+  <si>
+    <t>4 to 16 Positive Logic Decoder</t>
+  </si>
+  <si>
+    <t>MC14514BDWR2G</t>
+  </si>
+  <si>
+    <t>onsemi</t>
   </si>
 </sst>
 </file>
@@ -1772,6 +1781,10 @@
     </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
+<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -2096,7 +2109,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4BB64E12-2F57-4D15-BA8D-127B966BFCD4}">
-  <dimension ref="A1:R157"/>
+  <dimension ref="A1:R158"/>
   <sheetFormatPr defaultColWidth="11.44140625" defaultRowHeight="15.6" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="9.109375" style="3" customWidth="1"/>
@@ -2208,7 +2221,7 @@
     </row>
     <row r="6" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A6" s="3">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C6" s="3" t="s">
         <v>28</v>
@@ -2221,7 +2234,7 @@
       </c>
       <c r="J6" s="2">
         <f t="shared" ref="J6:J35" si="0">A6*I6</f>
-        <v>0.6</v>
+        <v>1.2</v>
       </c>
       <c r="K6" s="1" t="s">
         <v>447</v>
@@ -6866,6 +6879,39 @@
       <c r="J157" s="2">
         <f>A157*I157</f>
         <v>0</v>
+      </c>
+    </row>
+    <row r="158" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="A158" s="3">
+        <v>1</v>
+      </c>
+      <c r="C158" s="3" t="s">
+        <v>31</v>
+      </c>
+      <c r="D158" s="3" t="s">
+        <v>464</v>
+      </c>
+      <c r="E158" s="3" t="s">
+        <v>466</v>
+      </c>
+      <c r="F158" s="3" t="s">
+        <v>465</v>
+      </c>
+      <c r="G158" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="H158" s="3" t="s">
+        <v>465</v>
+      </c>
+      <c r="I158" s="2">
+        <v>1.1299999999999999</v>
+      </c>
+      <c r="J158" s="2">
+        <f>A158*I158</f>
+        <v>1.1299999999999999</v>
+      </c>
+      <c r="K158" s="1" t="s">
+        <v>195</v>
       </c>
     </row>
   </sheetData>

</xml_diff>